<commit_message>
Got TA, TR, PA, and PR surfplots working for speeds and RPMs
- Added assumption to Airfoil.m
Debugged in flightEnvelopeSizer quite a bit- marked the line with comment. Got TA, TR, PA, and PR surfplots working for speeds and RPMs
- Edited MotorPropAssy.m and Propeller.m to store data better: Propeller no longer stores missing data, and MotorPropAssy stores data for RPM values *through* the max RPM, not just at the max RPM
- Changed airfoil spreadsheets a bit to account for new assumption in Airfoil.m
</commit_message>
<xml_diff>
--- a/Propulsion & Power/Tabulated Airfoil c_d Values/E210_c_d.xlsx
+++ b/Propulsion & Power/Tabulated Airfoil c_d Values/E210_c_d.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mailmissouri-my.sharepoint.com/personal/arvkb9_umsystem_edu/Documents/896 - B.S Aerospace Engineering Courses/92 - Fall 2026/6 - AE4780-Meeks/Github Repo/Miner-Works-MW-27-MantaRay/Propulsion &amp; Power/Tabulated Airfoil c_d Values/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="8_{DC56BE96-02B0-466A-A13D-84E50E3BCDC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A71343D7-1EED-459D-BF38-7A18496A957B}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="8_{DC56BE96-02B0-466A-A13D-84E50E3BCDC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{60CE8171-43AE-409A-9B7E-93783D301BE9}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{706E62A6-5DB7-4E23-AC7D-EF51E1E871E8}"/>
   </bookViews>
@@ -886,7 +886,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{784AA86F-C3BA-47F6-A64C-FE3BBE194E9E}">
-  <dimension ref="A1:B71"/>
+  <dimension ref="A1:B37"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
@@ -1185,278 +1185,6 @@
         <v>1.528E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A38">
-        <v>9</v>
-      </c>
-      <c r="B38">
-        <v>1.7149999999999999E-2</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A39">
-        <v>9.5</v>
-      </c>
-      <c r="B39">
-        <v>1.9199999999999998E-2</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A40">
-        <v>10</v>
-      </c>
-      <c r="B40">
-        <v>2.1360000000000001E-2</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A41">
-        <v>10.5</v>
-      </c>
-      <c r="B41">
-        <v>2.419E-2</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A42">
-        <v>11</v>
-      </c>
-      <c r="B42">
-        <v>2.8539999999999999E-2</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A43">
-        <v>11.5</v>
-      </c>
-      <c r="B43">
-        <v>3.1919999999999997E-2</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A44">
-        <v>12</v>
-      </c>
-      <c r="B44">
-        <v>3.5830000000000001E-2</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A45">
-        <v>12.5</v>
-      </c>
-      <c r="B45">
-        <v>4.0390000000000002E-2</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A46">
-        <v>13</v>
-      </c>
-      <c r="B46">
-        <v>4.58E-2</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A47">
-        <v>13.5</v>
-      </c>
-      <c r="B47">
-        <v>5.203E-2</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A48">
-        <v>14</v>
-      </c>
-      <c r="B48">
-        <v>5.9560000000000002E-2</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A49">
-        <v>14.5</v>
-      </c>
-      <c r="B49">
-        <v>6.7720000000000002E-2</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A50">
-        <v>15</v>
-      </c>
-      <c r="B50">
-        <v>7.6660000000000006E-2</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A51">
-        <v>15.5</v>
-      </c>
-      <c r="B51">
-        <v>8.5720000000000005E-2</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A52">
-        <v>16</v>
-      </c>
-      <c r="B52">
-        <v>9.3840000000000007E-2</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A53">
-        <v>16.5</v>
-      </c>
-      <c r="B53">
-        <v>0.10199</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A54">
-        <v>17</v>
-      </c>
-      <c r="B54">
-        <v>0.10983999999999999</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A55">
-        <v>17.5</v>
-      </c>
-      <c r="B55">
-        <v>0.11876</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A56">
-        <v>18</v>
-      </c>
-      <c r="B56">
-        <v>0.13081000000000001</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A57">
-        <v>18.5</v>
-      </c>
-      <c r="B57">
-        <v>0.14565</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A58">
-        <v>19</v>
-      </c>
-      <c r="B58">
-        <v>0.16338</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A59">
-        <v>19.5</v>
-      </c>
-      <c r="B59">
-        <v>0.18486</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A60">
-        <v>20</v>
-      </c>
-      <c r="B60">
-        <v>0.21221999999999999</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A61">
-        <v>20.5</v>
-      </c>
-      <c r="B61">
-        <v>0.25879999999999997</v>
-      </c>
-    </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A62">
-        <v>21</v>
-      </c>
-      <c r="B62">
-        <v>0.29709000000000002</v>
-      </c>
-    </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A63">
-        <v>21.5</v>
-      </c>
-      <c r="B63">
-        <v>0.29593000000000003</v>
-      </c>
-    </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A64">
-        <v>22</v>
-      </c>
-      <c r="B64">
-        <v>0.29870999999999998</v>
-      </c>
-    </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A65">
-        <v>22.5</v>
-      </c>
-      <c r="B65">
-        <v>0.30230000000000001</v>
-      </c>
-    </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A66">
-        <v>23</v>
-      </c>
-      <c r="B66">
-        <v>0.30609999999999998</v>
-      </c>
-    </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A67">
-        <v>23.5</v>
-      </c>
-      <c r="B67">
-        <v>0.31080999999999998</v>
-      </c>
-    </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A68">
-        <v>24</v>
-      </c>
-      <c r="B68">
-        <v>0.31541000000000002</v>
-      </c>
-    </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A69">
-        <v>24.5</v>
-      </c>
-      <c r="B69">
-        <v>0.31931999999999999</v>
-      </c>
-    </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A70">
-        <v>25</v>
-      </c>
-      <c r="B70">
-        <v>0.32305</v>
-      </c>
-    </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A71">
-        <v>25.5</v>
-      </c>
-      <c r="B71">
-        <v>0.32661000000000001</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>